<commit_message>
Verifica settimanale: doppio controllo AI su 190 record (178 promossi), stato e log aggiornati
Doppio controllo indipendente (WebSearch, fonte diversa da quella già citata
in nota) sulle righe "DA VERIFICARE UMANAMENTE" nei 61 file nuovi non marcati
duplicati. 178 righe promosse a "VERIFICATA AI - doppio controllo
(14/09/2026)"; 12 lasciate invariate (9 per esito ambiguo/non confermato, 3
per incoerenza di settore nonostante esistenza aziendale confermata).
Nessuna riga declassata, nessuna riga cancellata.

Aggiornati weekly_verify_state.json (last_run_at, processed_files) e
weekly_verify_log.md con il riepilogo del run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014CgvovxTrdARiZ1ujqwH5a
</commit_message>
<xml_diff>
--- a/output/2026-09-07_15_Slovenia_Obalno-kraska_Metalworking_Lavorazioni_Metalliche.xlsx
+++ b/output/2026-09-07_15_Slovenia_Obalno-kraska_Metalworking_Lavorazioni_Metalliche.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (14/09/2026)</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (14/09/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>